<commit_message>
add hirachy to diagram_v7
</commit_message>
<xml_diff>
--- a/DB_related/inventory_2.xlsx
+++ b/DB_related/inventory_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\OneDrive\Documents\phecoding\dev-test1\test\DB_related\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAD6286A-4E00-476E-AE11-4A82299AFE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229D35EF-0E44-438C-95BA-9F842AE21269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{897BFD47-8918-48DA-A861-61C451B26815}"/>
+    <workbookView xWindow="780" yWindow="795" windowWidth="21600" windowHeight="11235" xr2:uid="{897BFD47-8918-48DA-A861-61C451B26815}"/>
   </bookViews>
   <sheets>
     <sheet name="102_mapping" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>sw</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t>g1/0/9</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Key 7 xxxx \n   Key 7 yyyyyyy    \n\n</t>
   </si>
 </sst>
 </file>
@@ -913,10 +919,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA00BE1F-8576-46BB-8D3C-83CA0954BB9A}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -929,8 +935,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>102</v>
       </c>
@@ -943,8 +952,11 @@
       <c r="D2" t="s">
         <v>6</v>
       </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>102</v>
       </c>
@@ -958,7 +970,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>102</v>
       </c>
@@ -972,7 +984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>102</v>
       </c>

</xml_diff>